<commit_message>
Datos de prueba: dos planes de desarrollo de ejemplo
Planes de Rocío Tamayo para Lorena Céspedes e Iván Restrepo, sobre sus
brechas reales en los datos de prueba. excel/planes-ejemplo.tsv trae las
mismas filas para pegarlas en el libro de OneDrive.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/CDP-Datos-prueba.xlsx
+++ b/excel/CDP-Datos-prueba.xlsx
@@ -179,8 +179,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="Planes" displayName="Planes" ref="A1:J2" headerRowCount="1">
-  <autoFilter ref="A1:J2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="Planes" displayName="Planes" ref="A1:J3" headerRowCount="1">
+  <autoFilter ref="A1:J3"/>
   <tableColumns count="10">
     <tableColumn id="1" name="id"/>
     <tableColumn id="2" name="persona_id"/>
@@ -58530,18 +58530,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
     <col width="8" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -58598,13 +58598,100 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>plan-ejemplo-lorena</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>lorena-cespedes</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Llevar la gestión de casos e incidentes a nivel avanzado</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Que en dos trimestres resuelva sin escalar los casos de complejidad media y lidere la comunicación de un incidente mayor de principio a fin.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>1. Acompañar a Camilo en la guardia de incidentes mayores durante un mes.
+2. Liderar la comunicación de un incidente con supervisión.
+3. Revisión mensual de 5 casos cerrados con su líder.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>f159,f149</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>rocio-tamayo</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>1767225600000</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1767225600000</v>
+      </c>
+      <c r="J2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>plan-ejemplo-ivan</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>ivan-restrepo</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Consolidar el nivel intermedio en casos y colaboración</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Que cierre los casos de primer nivel sin reabrirlos y documente cada solución para el resto del equipo.</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>1. Curso interno de gestión de casos.
+2. Documentar en la base de conocimiento cada caso que cierre durante un mes.
+3. Participar en la revisión semanal de casos del equipo.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>f159,f153</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>rocio-tamayo</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>1767225660000</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1767225660000</v>
+      </c>
+      <c r="J3" t="b">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>